<commit_message>
feature: mission system 추가.
</commit_message>
<xml_diff>
--- a/input/Domains/Game/MissionTable.xlsx
+++ b/input/Domains/Game/MissionTable.xlsx
@@ -2,29 +2,34 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="1420" yWindow="500" windowWidth="36980" windowHeight="21100" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="MISSION_DAILY" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="MISSION_WEEKLY" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="MISSION_ACHIEVEMENT" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="MISSION_ACHIEVE" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
-      <name val="Calibri"/>
+      <name val="맑은 고딕"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="맑은 고딕"/>
+      <charset val="129"/>
+      <family val="3"/>
+      <sz val="8"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -52,7 +57,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="표준" xfId="0" builtinId="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -415,8 +420,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G4"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:F4"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="17"/>
+  <cols>
+    <col width="18.5" bestFit="1" customWidth="1" min="1" max="1"/>
+    <col width="14.5" bestFit="1" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="3" max="6"/>
+    <col width="14.83203125" bestFit="1" customWidth="1" min="7" max="7"/>
+    <col width="21.1640625" bestFit="1" customWidth="1" min="8" max="8"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -436,22 +448,17 @@
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>conditionKey</t>
+          <t>conditionOp</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>conditionOp</t>
+          <t>conditionValue</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>conditionValue</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>rewardKey</t>
+          <t>rewardGroupId</t>
         </is>
       </c>
     </row>
@@ -468,25 +475,20 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>string</t>
+          <t>MISSION_CONDITION_TYPE</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>string</t>
+          <t>MISSION_OP_TYPE</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>string</t>
+          <t>class:CBigInt</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
-        <is>
-          <t>int</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
         <is>
           <t>string</t>
         </is>
@@ -498,12 +500,6 @@
           <t>pk</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr"/>
-      <c r="C3" t="inlineStr"/>
-      <c r="D3" t="inlineStr"/>
-      <c r="E3" t="inlineStr"/>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -518,27 +514,22 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>조건 타입(예: StatAtLeast, CountAtLeast)</t>
+          <t>미션 조건 타입 enum (MissionConditionType, source: ENUM_TYPES.json)</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>조건 키(예: stage_clear_count)</t>
+          <t>미션 진행 연산 enum (MissionOpType, MAX/SUM/TOTAL)</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>연산자 표현(예: &gt;=)</t>
+          <t>조건 목표값 (CBigInt, plain format: {base, pow}, 예: {5.5, 6})</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>목표값</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>RewardKey (정본)</t>
+          <t>RewardGroupId (정본)</t>
         </is>
       </c>
     </row>
@@ -553,78 +544,96 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G4"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:H4"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="17"/>
+  <cols>
+    <col width="11.83203125" bestFit="1" customWidth="1" min="1" max="1"/>
+    <col width="18.5" bestFit="1" customWidth="1" min="2" max="2"/>
+    <col width="14.5" bestFit="1" customWidth="1" min="3" max="3"/>
+    <col width="14.5" customWidth="1" min="4" max="4"/>
+    <col width="25.33203125" customWidth="1" min="5" max="8"/>
+    <col width="21.1640625" bestFit="1" customWidth="1" min="9" max="9"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
+          <t>index</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
           <t>missionId</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>isActive</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>level</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
         <is>
           <t>conditionType</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>conditionKey</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>conditionOp</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>conditionValue</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>rewardKey</t>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>rewardGroupId</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
+          <t>int</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
           <t>string</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>bool</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>string</t>
-        </is>
-      </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>string</t>
+          <t>int</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>string</t>
+          <t>MISSION_CONDITION_TYPE</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>int</t>
+          <t>MISSION_OP_TYPE</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
+        <is>
+          <t>class:CBigInt</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
         <is>
           <t>string</t>
         </is>
@@ -636,185 +645,41 @@
           <t>pk</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr"/>
-      <c r="C3" t="inlineStr"/>
-      <c r="D3" t="inlineStr"/>
-      <c r="E3" t="inlineStr"/>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr"/>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>group:true</t>
+        </is>
+      </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="B4" t="inlineStr">
         <is>
           <t>내부 미션 ID (정본)</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="C4" t="inlineStr">
         <is>
           <t>운영 활성 토글</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>조건 타입(예: StatAtLeast, CountAtLeast)</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>조건 키(예: stage_clear_count)</t>
-        </is>
-      </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>연산자 표현(예: &gt;=)</t>
+          <t>미션 조건 타입 enum (MissionConditionType, source: ENUM_TYPES.json)</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>목표값</t>
+          <t>미션 진행 연산 enum (MissionOpType, MAX/SUM/TOTAL)</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>RewardKey (정본)</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:G4"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>missionId</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>isActive</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>conditionType</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>conditionKey</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>conditionOp</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>conditionValue</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>rewardKey</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>string</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>bool</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>string</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>string</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>string</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>int</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>string</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>pk</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr"/>
-      <c r="C3" t="inlineStr"/>
-      <c r="D3" t="inlineStr"/>
-      <c r="E3" t="inlineStr"/>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr"/>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>내부 미션 ID (정본)</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>운영 활성 토글</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>조건 타입(예: StatAtLeast, CountAtLeast)</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>조건 키(예: stage_clear_count)</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>연산자 표현(예: &gt;=)</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>목표값</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>RewardKey (정본)</t>
+          <t>조건 목표값 (CBigInt, plain format: {base, pow}, 예: {5.5, 6})</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>RewardGroupId (정본)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: 누락된 test data 추가.
</commit_message>
<xml_diff>
--- a/input/Domains/Game/MissionTable.xlsx
+++ b/input/Domains/Game/MissionTable.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/maoshy/Documents/Projects/devian/input/Domains/Game/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B2BBB7A-67C1-1C4A-B718-D551E6635298}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D5CFFF23-71D8-204B-ADAB-64C24BB4A377}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1420" yWindow="500" windowWidth="36980" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1420" yWindow="500" windowWidth="36980" windowHeight="21100" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="MISSION_DAILY" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="117" uniqueCount="65">
   <si>
     <t>missionId</t>
   </si>
@@ -122,96 +122,114 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
+    <t>{100, 0}</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>{300, 0}</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>{1000, 0}</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>{5000, 0}</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>{30000, 0}</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>{4, 0}</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>{5, 0}</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>reward_mission_day_001</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>reward_mission_day_002</t>
+  </si>
+  <si>
+    <t>reward_mission_day_003</t>
+  </si>
+  <si>
+    <t>reward_mission_day_004</t>
+  </si>
+  <si>
+    <t>reward_mission_day_005</t>
+  </si>
+  <si>
+    <t>reward_mission_achieve_001</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>reward_mission_achieve_002</t>
+  </si>
+  <si>
+    <t>reward_mission_achieve_003</t>
+  </si>
+  <si>
+    <t>reward_mission_achieve_004</t>
+  </si>
+  <si>
+    <t>reward_mission_achieve_005</t>
+  </si>
+  <si>
+    <t>TEST_001</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>TEST_002</t>
+  </si>
+  <si>
+    <t>TEST_003</t>
+  </si>
+  <si>
+    <t>TEST_004</t>
+  </si>
+  <si>
+    <t>MISSION_CLEAR</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>TEST_005</t>
+  </si>
+  <si>
+    <t>mission_achieve_001</t>
+  </si>
+  <si>
     <t>mission_achieve_002</t>
   </si>
   <si>
+    <t>TEST_006</t>
+  </si>
+  <si>
     <t>mission_achieve_003</t>
   </si>
   <si>
+    <t>TEST_007</t>
+  </si>
+  <si>
     <t>mission_achieve_004</t>
   </si>
   <si>
+    <t>TEST_008</t>
+  </si>
+  <si>
+    <t>{100, 0}</t>
+  </si>
+  <si>
     <t>mission_achieve_005</t>
   </si>
   <si>
-    <t>{100, 0}</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>{300, 0}</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>{1000, 0}</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>{5000, 0}</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>{30000, 0}</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>{4, 0}</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>{5, 0}</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>reward_mission_day_001</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>reward_mission_day_002</t>
-  </si>
-  <si>
-    <t>reward_mission_day_003</t>
-  </si>
-  <si>
-    <t>reward_mission_day_004</t>
-  </si>
-  <si>
-    <t>reward_mission_day_005</t>
-  </si>
-  <si>
-    <t>reward_mission_achieve_001</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>reward_mission_achieve_002</t>
-  </si>
-  <si>
-    <t>reward_mission_achieve_003</t>
-  </si>
-  <si>
-    <t>reward_mission_achieve_004</t>
-  </si>
-  <si>
-    <t>reward_mission_achieve_005</t>
-  </si>
-  <si>
-    <t>TEST_001</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>TEST_002</t>
-  </si>
-  <si>
-    <t>TEST_003</t>
-  </si>
-  <si>
-    <t>TEST_004</t>
-  </si>
-  <si>
-    <t>MISSION_CLEAR</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>TEST_005</t>
+    <t>TEST_009</t>
   </si>
 </sst>
 </file>
@@ -653,16 +671,16 @@
         <v>1</v>
       </c>
       <c r="D5" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="E5" t="s">
         <v>30</v>
       </c>
       <c r="F5" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="G5" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
     </row>
     <row r="6" spans="1:7">
@@ -673,16 +691,16 @@
         <v>1</v>
       </c>
       <c r="D6" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="E6" t="s">
         <v>30</v>
       </c>
       <c r="F6" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="G6" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
     </row>
     <row r="7" spans="1:7">
@@ -693,16 +711,16 @@
         <v>1</v>
       </c>
       <c r="D7" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="E7" t="s">
         <v>30</v>
       </c>
       <c r="F7" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="G7" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
     </row>
     <row r="8" spans="1:7">
@@ -713,16 +731,16 @@
         <v>1</v>
       </c>
       <c r="D8" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="E8" t="s">
         <v>30</v>
       </c>
       <c r="F8" t="s">
+        <v>38</v>
+      </c>
+      <c r="G8" t="s">
         <v>42</v>
-      </c>
-      <c r="G8" t="s">
-        <v>46</v>
       </c>
     </row>
     <row r="9" spans="1:7">
@@ -733,16 +751,16 @@
         <v>1</v>
       </c>
       <c r="D9" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="E9" t="s">
         <v>30</v>
       </c>
       <c r="F9" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="G9" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
     </row>
   </sheetData>
@@ -753,7 +771,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:H9"/>
+  <dimension ref="A1:H13"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="17"/>
   <cols>
     <col min="1" max="1" width="11.83203125" bestFit="1" customWidth="1"/>
@@ -861,16 +879,16 @@
         <v>1</v>
       </c>
       <c r="E5" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="F5" t="s">
         <v>30</v>
       </c>
       <c r="G5" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="H5" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -878,7 +896,7 @@
         <v>2</v>
       </c>
       <c r="B6" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C6" t="b">
         <v>1</v>
@@ -887,16 +905,16 @@
         <v>2</v>
       </c>
       <c r="E6" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="F6" t="s">
         <v>30</v>
       </c>
       <c r="G6" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="H6" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
     </row>
     <row r="7" spans="1:8">
@@ -904,7 +922,7 @@
         <v>3</v>
       </c>
       <c r="B7" t="s">
-        <v>33</v>
+        <v>55</v>
       </c>
       <c r="C7" t="b">
         <v>1</v>
@@ -913,16 +931,16 @@
         <v>3</v>
       </c>
       <c r="E7" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="F7" t="s">
         <v>30</v>
       </c>
       <c r="G7" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="H7" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -930,7 +948,7 @@
         <v>4</v>
       </c>
       <c r="B8" t="s">
-        <v>34</v>
+        <v>55</v>
       </c>
       <c r="C8" t="b">
         <v>1</v>
@@ -939,16 +957,16 @@
         <v>4</v>
       </c>
       <c r="E8" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="F8" t="s">
         <v>30</v>
       </c>
       <c r="G8" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="H8" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
     </row>
     <row r="9" spans="1:8">
@@ -956,7 +974,7 @@
         <v>5</v>
       </c>
       <c r="B9" t="s">
-        <v>35</v>
+        <v>55</v>
       </c>
       <c r="C9" t="b">
         <v>1</v>
@@ -965,16 +983,120 @@
         <v>5</v>
       </c>
       <c r="E9" t="s">
+        <v>54</v>
+      </c>
+      <c r="F9" t="s">
+        <v>30</v>
+      </c>
+      <c r="G9" t="s">
+        <v>36</v>
+      </c>
+      <c r="H9" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8">
+      <c r="A10">
+        <v>6</v>
+      </c>
+      <c r="B10" t="s">
+        <v>56</v>
+      </c>
+      <c r="C10" t="b">
+        <v>1</v>
+      </c>
+      <c r="D10">
+        <v>1</v>
+      </c>
+      <c r="E10" t="s">
+        <v>57</v>
+      </c>
+      <c r="F10" t="s">
+        <v>30</v>
+      </c>
+      <c r="G10" t="s">
+        <v>32</v>
+      </c>
+      <c r="H10" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8">
+      <c r="A11">
+        <v>7</v>
+      </c>
+      <c r="B11" t="s">
         <v>58</v>
       </c>
-      <c r="F9" t="s">
-        <v>30</v>
-      </c>
-      <c r="G9" t="s">
-        <v>40</v>
-      </c>
-      <c r="H9" t="s">
-        <v>52</v>
+      <c r="C11" t="b">
+        <v>1</v>
+      </c>
+      <c r="D11">
+        <v>1</v>
+      </c>
+      <c r="E11" t="s">
+        <v>59</v>
+      </c>
+      <c r="F11" t="s">
+        <v>30</v>
+      </c>
+      <c r="G11" t="s">
+        <v>32</v>
+      </c>
+      <c r="H11" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8">
+      <c r="A12">
+        <v>8</v>
+      </c>
+      <c r="B12" t="s">
+        <v>60</v>
+      </c>
+      <c r="C12" t="b">
+        <v>1</v>
+      </c>
+      <c r="D12">
+        <v>1</v>
+      </c>
+      <c r="E12" t="s">
+        <v>61</v>
+      </c>
+      <c r="F12" t="s">
+        <v>30</v>
+      </c>
+      <c r="G12" t="s">
+        <v>62</v>
+      </c>
+      <c r="H12" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8">
+      <c r="A13">
+        <v>9</v>
+      </c>
+      <c r="B13" t="s">
+        <v>63</v>
+      </c>
+      <c r="C13" t="b">
+        <v>1</v>
+      </c>
+      <c r="D13">
+        <v>1</v>
+      </c>
+      <c r="E13" t="s">
+        <v>64</v>
+      </c>
+      <c r="F13" t="s">
+        <v>30</v>
+      </c>
+      <c r="G13" t="s">
+        <v>62</v>
+      </c>
+      <c r="H13" t="s">
+        <v>48</v>
       </c>
     </row>
   </sheetData>

</xml_diff>